<commit_message>
templates: regenerate MFRS SOFP/SOPL formulas from linkbase
Regenerate face/sub rollup formulas for the MFRS SOFP and SOPL templates
(Company + Group) via scripts/regenerate_mfrs_sofp_sopl_formulas.py.
Snapshot the pre-regeneration templates under
archive-2026-04-28-pre-linkbase-regeneration/ and capture the before/after
in docs/template-formula-change-audit-2026-05-22.md per gotcha #3.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XBRL-template-MFRS/Company/01-SOFP-CuNonCu.xlsx
+++ b/XBRL-template-MFRS/Company/01-SOFP-CuNonCu.xlsx
@@ -641,6 +641,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1" s="13">
       <c r="A3" s="30" t="inlineStr">
         <is>
@@ -1082,11 +1083,11 @@
         </is>
       </c>
       <c r="B37" s="38">
-        <f>1*B8+1*B9+1*B11+1*B12+1*B13+1*B14+1*B15+1*B16+1*B17+1*B18+1*B19+1*B20+1*B21+1*B22+1*B25+1*B27+1*B28+1*B29+1*B30+1*B31+1*B32+1*B33+1*B35+1*B26+1*B10</f>
+        <f>1*B8+1*B9+1*B10+1*B11+1*B12+1*B13+1*B14+1*B15+1*B16+1*B17+1*B18+1*B19+1*B20+1*B21+1*B22+1*B25+1*B26+1*B27+1*B28+1*B29+1*B30+1*B31+1*B32+1*B33+1*B35</f>
         <v/>
       </c>
       <c r="C37" s="38">
-        <f>1*C8+1*C9+1*C11+1*C12+1*C13+1*C14+1*C15+1*C16+1*C17+1*C18+1*C19+1*C20+1*C21+1*C22+1*C25+1*C27+1*C28+1*C29+1*C30+1*C31+1*C32+1*C33+1*C35+1*C26+1*C10</f>
+        <f>1*C8+1*C9+1*C10+1*C11+1*C12+1*C13+1*C14+1*C15+1*C16+1*C17+1*C18+1*C19+1*C20+1*C21+1*C22+1*C25+1*C26+1*C27+1*C28+1*C29+1*C30+1*C31+1*C32+1*C33+1*C35</f>
         <v/>
       </c>
       <c r="D37" s="43" t="n"/>
@@ -1566,11 +1567,11 @@
         </is>
       </c>
       <c r="B74" s="38">
-        <f>1*B60+1*B73</f>
+        <f>1*B50+1*B51+1*B52+1*B53+1*B54+1*B55+1*B56+1*B57+1*B58+1*B59+1*B62+1*B63+1*B64+1*B65+1*B66+1*B67+1*B68+1*B69+1*B70+1*B72</f>
         <v/>
       </c>
       <c r="C74" s="38">
-        <f>1*C60+1*C73</f>
+        <f>1*C50+1*C51+1*C52+1*C53+1*C54+1*C55+1*C56+1*C57+1*C58+1*C59+1*C62+1*C63+1*C64+1*C65+1*C66+1*C67+1*C68+1*C69+1*C70+1*C72</f>
         <v/>
       </c>
       <c r="D74" s="43" t="n"/>
@@ -1630,6 +1631,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1" s="13">
       <c r="A3" s="30" t="inlineStr">
         <is>
@@ -3955,11 +3957,11 @@
         </is>
       </c>
       <c r="B214" s="38">
-        <f>1*B206+1*B207+1*B208+1*B209+1*B210+1*B211+1*B213+1*B212</f>
+        <f>1*B206+1*B207+1*B208+1*B209+1*B210+1*B211+1*B212+1*B213</f>
         <v/>
       </c>
       <c r="C214" s="38">
-        <f>1*C206+1*C207+1*C208+1*C209+1*C210+1*C211+1*C213+1*C212</f>
+        <f>1*C206+1*C207+1*C208+1*C209+1*C210+1*C211+1*C212+1*C213</f>
         <v/>
       </c>
       <c r="D214" s="43" t="n"/>
@@ -4487,11 +4489,11 @@
         </is>
       </c>
       <c r="B263" s="38">
-        <f>1*B278+1*B259+1*B260+1*B261+1*B262</f>
+        <f>1*B258+1*B259+1*B260+1*B261+1*B262</f>
         <v/>
       </c>
       <c r="C263" s="38">
-        <f>1*C278+1*C259+1*C260+1*C261+1*C262</f>
+        <f>1*C258+1*C259+1*C260+1*C261+1*C262</f>
         <v/>
       </c>
       <c r="D263" s="43" t="n"/>
@@ -5623,11 +5625,11 @@
         </is>
       </c>
       <c r="B367" s="38">
-        <f>1*B382+1*B363+1*B364+1*B365+1*B366</f>
+        <f>1*B362+1*B363+1*B364+1*B365+1*B366</f>
         <v/>
       </c>
       <c r="C367" s="38">
-        <f>1*C382+1*C363+1*C364+1*C365+1*C366</f>
+        <f>1*C362+1*C363+1*C364+1*C365+1*C366</f>
         <v/>
       </c>
       <c r="D367" s="43" t="n"/>
@@ -5699,11 +5701,11 @@
         </is>
       </c>
       <c r="B374" s="38">
-        <f>1*B389+1*B370+1*B371+1*B372+1*B373</f>
+        <f>1*B369+1*B370+1*B371+1*B372+1*B373</f>
         <v/>
       </c>
       <c r="C374" s="38">
-        <f>1*C389+1*C370+1*C371+1*C372+1*C373</f>
+        <f>1*C369+1*C370+1*C371+1*C372+1*C373</f>
         <v/>
       </c>
       <c r="D374" s="43" t="n"/>
@@ -5801,11 +5803,11 @@
         </is>
       </c>
       <c r="B383" s="38">
-        <f>1*B349+1*B360+1*B387+1*B394+1*B382</f>
+        <f>1*B349+1*B360+1*B367+1*B374+1*B382</f>
         <v/>
       </c>
       <c r="C383" s="38">
-        <f>1*C349+1*C360+1*C387+1*C394+1*C382</f>
+        <f>1*C349+1*C360+1*C367+1*C374+1*C382</f>
         <v/>
       </c>
       <c r="D383" s="43" t="n"/>

</xml_diff>